<commit_message>
Add usage data for 24 and 26 Oct 2026 (3 + 11 logins); merge 1 late 23 Oct login
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/daily_snapshots/Daily Usage Snapshot - 23-10-2026.xlsx
+++ b/daily_snapshots/Daily Usage Snapshot - 23-10-2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -787,6 +787,57 @@
         </is>
       </c>
       <c r="I8" t="inlineStr">
+        <is>
+          <t>Paying</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>user1787556989.3403</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ginabelletjie@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Gina</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Wright</t>
+        </is>
+      </c>
+      <c r="E9">
+        <f>_xlfn.CONCAT(C16:D16)</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Teacher</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Friday, 23 October 2026 at 16:59</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Applewood Preparatory</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Classroom</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>Paying</t>
         </is>

</xml_diff>

<commit_message>
Add Sponsored Schools lifetime section (AC Pipeline 10)
- update_sales_dashboard.py writes sponsored_schools.json from Pipeline 10
  (Approved - Onboarding, Renewal Review, Active - Sponsored; ZAR; not lost)
- update_dashboard.py renders a second lifetime-activity chart for them and
  lists them separately in the daily report instead of INVESTIGATE
- Alias fixes for Sun Valley and York High George
- Realign one 23 Oct row merged from an export with an extra column
- Renewals: Generation Schools Hermanus invoice paid

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/daily_snapshots/Daily Usage Snapshot - 23-10-2026.xlsx
+++ b/daily_snapshots/Daily Usage Snapshot - 23-10-2026.xlsx
@@ -813,31 +813,27 @@
           <t>Wright</t>
         </is>
       </c>
-      <c r="E9">
-        <f>_xlfn.CONCAT(C16:D16)</f>
-        <v/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Teacher</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Friday, 23 October 2026 at 16:59</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Friday, 23 October 2026 at 16:59</t>
+          <t>Applewood Preparatory</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Applewood Preparatory</t>
+          <t>Classroom</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
-        <is>
-          <t>Classroom</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
         <is>
           <t>Paying</t>
         </is>

</xml_diff>